<commit_message>
Add Razorpay billing and fix reported document workflows
</commit_message>
<xml_diff>
--- a/frontend/public/templates/BreezyInvoice-employee-import-template.xlsx
+++ b/frontend/public/templates/BreezyInvoice-employee-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R5a3ab003653e48af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="2" r:id="Ra2135915e56146f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R9dcb144175994e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="2" r:id="Rd481e0afb59041f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -276,26 +276,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EmployeeImportTable" displayName="EmployeeImportTable" ref="A1:R52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="18">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EmployeeImportTable" displayName="EmployeeImportTable" ref="A1:S200" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="Employee Code"/>
     <x:tableColumn id="2" name="Employee Name"/>
-    <x:tableColumn id="3" name="Designation"/>
-    <x:tableColumn id="4" name="Department"/>
-    <x:tableColumn id="5" name="PAN"/>
-    <x:tableColumn id="6" name="UAN"/>
-    <x:tableColumn id="7" name="ESI Number"/>
-    <x:tableColumn id="8" name="Bank Name"/>
-    <x:tableColumn id="9" name="Bank Account Number"/>
-    <x:tableColumn id="10" name="IFSC"/>
-    <x:tableColumn id="11" name="Employment Status"/>
-    <x:tableColumn id="12" name="Joining Date"/>
-    <x:tableColumn id="13" name="Basic Salary"/>
-    <x:tableColumn id="14" name="HRA"/>
-    <x:tableColumn id="15" name="Special Allowance"/>
-    <x:tableColumn id="16" name="PF"/>
-    <x:tableColumn id="17" name="Professional Tax"/>
-    <x:tableColumn id="18" name="TDS"/>
+    <x:tableColumn id="3" name="Email"/>
+    <x:tableColumn id="4" name="Designation"/>
+    <x:tableColumn id="5" name="Department"/>
+    <x:tableColumn id="6" name="PAN"/>
+    <x:tableColumn id="7" name="UAN"/>
+    <x:tableColumn id="8" name="ESI Number"/>
+    <x:tableColumn id="9" name="Bank Name"/>
+    <x:tableColumn id="10" name="Bank Account Number"/>
+    <x:tableColumn id="11" name="IFSC"/>
+    <x:tableColumn id="12" name="Employment Status"/>
+    <x:tableColumn id="13" name="Joining Date"/>
+    <x:tableColumn id="14" name="Basic Salary"/>
+    <x:tableColumn id="15" name="HRA"/>
+    <x:tableColumn id="16" name="Special Allowance"/>
+    <x:tableColumn id="17" name="PF"/>
+    <x:tableColumn id="18" name="Professional Tax"/>
+    <x:tableColumn id="19" name="TDS"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -669,7 +670,7 @@
   <x:cols>
     <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
@@ -695,51 +696,54 @@
         <x:v>Employee Name</x:v>
       </x:c>
       <x:c r="C1" s="25" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="D1" s="25" t="str">
         <x:v>Designation</x:v>
       </x:c>
-      <x:c r="D1" s="25" t="str">
+      <x:c r="E1" s="25" t="str">
         <x:v>Department</x:v>
       </x:c>
-      <x:c r="E1" s="25" t="str">
+      <x:c r="F1" s="25" t="str">
         <x:v>PAN</x:v>
       </x:c>
-      <x:c r="F1" s="25" t="str">
+      <x:c r="G1" s="25" t="str">
         <x:v>UAN</x:v>
       </x:c>
-      <x:c r="G1" s="25" t="str">
+      <x:c r="H1" s="25" t="str">
         <x:v>ESI Number</x:v>
       </x:c>
-      <x:c r="H1" s="25" t="str">
+      <x:c r="I1" s="25" t="str">
         <x:v>Bank Name</x:v>
       </x:c>
-      <x:c r="I1" s="25" t="str">
+      <x:c r="J1" s="25" t="str">
         <x:v>Bank Account Number</x:v>
       </x:c>
-      <x:c r="J1" s="25" t="str">
+      <x:c r="K1" s="25" t="str">
         <x:v>IFSC</x:v>
       </x:c>
-      <x:c r="K1" s="25" t="str">
+      <x:c r="L1" s="25" t="str">
         <x:v>Employment Status</x:v>
       </x:c>
-      <x:c r="L1" s="25" t="str">
+      <x:c r="M1" s="25" t="str">
         <x:v>Joining Date</x:v>
       </x:c>
-      <x:c r="M1" s="25" t="str">
+      <x:c r="N1" s="25" t="str">
         <x:v>Basic Salary</x:v>
       </x:c>
-      <x:c r="N1" s="25" t="str">
+      <x:c r="O1" s="25" t="str">
         <x:v>HRA</x:v>
       </x:c>
-      <x:c r="O1" s="25" t="str">
+      <x:c r="P1" s="25" t="str">
         <x:v>Special Allowance</x:v>
       </x:c>
-      <x:c r="P1" s="25" t="str">
+      <x:c r="Q1" s="25" t="str">
         <x:v>PF</x:v>
       </x:c>
-      <x:c r="Q1" s="25" t="str">
+      <x:c r="R1" s="25" t="str">
         <x:v>Professional Tax</x:v>
       </x:c>
-      <x:c r="R1" s="25" t="str">
+      <x:c r="S1" t="str">
         <x:v>TDS</x:v>
       </x:c>
     </x:row>
@@ -751,52 +755,55 @@
         <x:v>Rahul Sharma</x:v>
       </x:c>
       <x:c r="C2" s="34" t="str">
+        <x:v>rahul@example.com</x:v>
+      </x:c>
+      <x:c r="D2" s="34" t="str">
         <x:v>Accounts Executive</x:v>
       </x:c>
-      <x:c r="D2" s="34" t="str">
+      <x:c r="E2" s="34" t="str">
         <x:v>Finance</x:v>
       </x:c>
-      <x:c r="E2" s="34" t="str">
+      <x:c r="F2" s="34" t="str">
         <x:v>ABCDE1234F</x:v>
       </x:c>
-      <x:c r="F2" s="34" t="str"/>
-      <x:c r="G2" s="34" t="str"/>
-      <x:c r="H2" s="34" t="str">
+      <x:c r="G2" s="34"/>
+      <x:c r="H2" s="34"/>
+      <x:c r="I2" s="34" t="str">
         <x:v>HDFC Bank</x:v>
       </x:c>
-      <x:c r="I2" s="34" t="str"/>
-      <x:c r="J2" s="34" t="str">
+      <x:c r="J2" s="34"/>
+      <x:c r="K2" s="34" t="str">
         <x:v>HDFC0001234</x:v>
       </x:c>
-      <x:c r="K2" s="34" t="str">
+      <x:c r="L2" s="34" t="str">
         <x:v>Regular Full-time</x:v>
       </x:c>
-      <x:c r="L2" s="34" t="str">
+      <x:c r="M2" s="42" t="str">
         <x:v>2026-04-01</x:v>
       </x:c>
-      <x:c r="M2" s="42" t="n">
+      <x:c r="N2" s="42" t="n">
         <x:v>30000</x:v>
       </x:c>
-      <x:c r="N2" s="42" t="n">
+      <x:c r="O2" s="42" t="n">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="O2" s="42" t="n">
+      <x:c r="P2" s="42" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="P2" s="42" t="n">
+      <x:c r="Q2" s="42" t="n">
         <x:v>3600</x:v>
       </x:c>
-      <x:c r="Q2" s="42" t="n">
+      <x:c r="R2" s="42" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="R2" s="42" t="n">
+      <x:c r="S2" t="n">
         <x:v>1500</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="35"/>
       <x:c r="B3" s="36"/>
-      <x:c r="C3" s="36"/>
+      <x:c r="C3" s="36" t="str"/>
       <x:c r="D3" s="36"/>
       <x:c r="E3" s="36"/>
       <x:c r="F3" s="36"/>
@@ -812,11 +819,12 @@
       <x:c r="P3" s="43"/>
       <x:c r="Q3" s="43"/>
       <x:c r="R3" s="44"/>
+      <x:c r="S3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="37"/>
       <x:c r="B4" s="38"/>
-      <x:c r="C4" s="38"/>
+      <x:c r="C4" s="38" t="str"/>
       <x:c r="D4" s="38"/>
       <x:c r="E4" s="38"/>
       <x:c r="F4" s="38"/>
@@ -832,11 +840,12 @@
       <x:c r="P4" s="45"/>
       <x:c r="Q4" s="45"/>
       <x:c r="R4" s="46"/>
+      <x:c r="S4"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="37"/>
       <x:c r="B5" s="38"/>
-      <x:c r="C5" s="38"/>
+      <x:c r="C5" s="38" t="str"/>
       <x:c r="D5" s="38"/>
       <x:c r="E5" s="38"/>
       <x:c r="F5" s="38"/>
@@ -852,11 +861,12 @@
       <x:c r="P5" s="45"/>
       <x:c r="Q5" s="45"/>
       <x:c r="R5" s="46"/>
+      <x:c r="S5"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="37"/>
       <x:c r="B6" s="38"/>
-      <x:c r="C6" s="38"/>
+      <x:c r="C6" s="38" t="str"/>
       <x:c r="D6" s="38"/>
       <x:c r="E6" s="38"/>
       <x:c r="F6" s="38"/>
@@ -872,11 +882,12 @@
       <x:c r="P6" s="45"/>
       <x:c r="Q6" s="45"/>
       <x:c r="R6" s="46"/>
+      <x:c r="S6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="37"/>
       <x:c r="B7" s="38"/>
-      <x:c r="C7" s="38"/>
+      <x:c r="C7" s="38" t="str"/>
       <x:c r="D7" s="38"/>
       <x:c r="E7" s="38"/>
       <x:c r="F7" s="38"/>
@@ -892,11 +903,12 @@
       <x:c r="P7" s="45"/>
       <x:c r="Q7" s="45"/>
       <x:c r="R7" s="46"/>
+      <x:c r="S7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="37"/>
       <x:c r="B8" s="38"/>
-      <x:c r="C8" s="38"/>
+      <x:c r="C8" s="38" t="str"/>
       <x:c r="D8" s="38"/>
       <x:c r="E8" s="38"/>
       <x:c r="F8" s="38"/>
@@ -912,11 +924,12 @@
       <x:c r="P8" s="45"/>
       <x:c r="Q8" s="45"/>
       <x:c r="R8" s="46"/>
+      <x:c r="S8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="37"/>
       <x:c r="B9" s="38"/>
-      <x:c r="C9" s="38"/>
+      <x:c r="C9" s="38" t="str"/>
       <x:c r="D9" s="38"/>
       <x:c r="E9" s="38"/>
       <x:c r="F9" s="38"/>
@@ -932,11 +945,12 @@
       <x:c r="P9" s="45"/>
       <x:c r="Q9" s="45"/>
       <x:c r="R9" s="46"/>
+      <x:c r="S9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="37"/>
       <x:c r="B10" s="38"/>
-      <x:c r="C10" s="38"/>
+      <x:c r="C10" s="38" t="str"/>
       <x:c r="D10" s="38"/>
       <x:c r="E10" s="38"/>
       <x:c r="F10" s="38"/>
@@ -952,11 +966,12 @@
       <x:c r="P10" s="45"/>
       <x:c r="Q10" s="45"/>
       <x:c r="R10" s="46"/>
+      <x:c r="S10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="37"/>
       <x:c r="B11" s="38"/>
-      <x:c r="C11" s="38"/>
+      <x:c r="C11" s="38" t="str"/>
       <x:c r="D11" s="38"/>
       <x:c r="E11" s="38"/>
       <x:c r="F11" s="38"/>
@@ -972,11 +987,12 @@
       <x:c r="P11" s="45"/>
       <x:c r="Q11" s="45"/>
       <x:c r="R11" s="46"/>
+      <x:c r="S11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="37"/>
       <x:c r="B12" s="38"/>
-      <x:c r="C12" s="38"/>
+      <x:c r="C12" s="38" t="str"/>
       <x:c r="D12" s="38"/>
       <x:c r="E12" s="38"/>
       <x:c r="F12" s="38"/>
@@ -992,11 +1008,12 @@
       <x:c r="P12" s="45"/>
       <x:c r="Q12" s="45"/>
       <x:c r="R12" s="46"/>
+      <x:c r="S12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="37"/>
       <x:c r="B13" s="38"/>
-      <x:c r="C13" s="38"/>
+      <x:c r="C13" s="38" t="str"/>
       <x:c r="D13" s="38"/>
       <x:c r="E13" s="38"/>
       <x:c r="F13" s="38"/>
@@ -1012,11 +1029,12 @@
       <x:c r="P13" s="45"/>
       <x:c r="Q13" s="45"/>
       <x:c r="R13" s="46"/>
+      <x:c r="S13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="37"/>
       <x:c r="B14" s="38"/>
-      <x:c r="C14" s="38"/>
+      <x:c r="C14" s="38" t="str"/>
       <x:c r="D14" s="38"/>
       <x:c r="E14" s="38"/>
       <x:c r="F14" s="38"/>
@@ -1032,11 +1050,12 @@
       <x:c r="P14" s="45"/>
       <x:c r="Q14" s="45"/>
       <x:c r="R14" s="46"/>
+      <x:c r="S14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="37"/>
       <x:c r="B15" s="38"/>
-      <x:c r="C15" s="38"/>
+      <x:c r="C15" s="38" t="str"/>
       <x:c r="D15" s="38"/>
       <x:c r="E15" s="38"/>
       <x:c r="F15" s="38"/>
@@ -1052,11 +1071,12 @@
       <x:c r="P15" s="45"/>
       <x:c r="Q15" s="45"/>
       <x:c r="R15" s="46"/>
+      <x:c r="S15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="37"/>
       <x:c r="B16" s="38"/>
-      <x:c r="C16" s="38"/>
+      <x:c r="C16" s="38" t="str"/>
       <x:c r="D16" s="38"/>
       <x:c r="E16" s="38"/>
       <x:c r="F16" s="38"/>
@@ -1072,11 +1092,12 @@
       <x:c r="P16" s="45"/>
       <x:c r="Q16" s="45"/>
       <x:c r="R16" s="46"/>
+      <x:c r="S16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="37"/>
       <x:c r="B17" s="38"/>
-      <x:c r="C17" s="38"/>
+      <x:c r="C17" s="38" t="str"/>
       <x:c r="D17" s="38"/>
       <x:c r="E17" s="38"/>
       <x:c r="F17" s="38"/>
@@ -1092,11 +1113,12 @@
       <x:c r="P17" s="45"/>
       <x:c r="Q17" s="45"/>
       <x:c r="R17" s="46"/>
+      <x:c r="S17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="37"/>
       <x:c r="B18" s="38"/>
-      <x:c r="C18" s="38"/>
+      <x:c r="C18" s="38" t="str"/>
       <x:c r="D18" s="38"/>
       <x:c r="E18" s="38"/>
       <x:c r="F18" s="38"/>
@@ -1112,11 +1134,12 @@
       <x:c r="P18" s="45"/>
       <x:c r="Q18" s="45"/>
       <x:c r="R18" s="46"/>
+      <x:c r="S18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="37"/>
       <x:c r="B19" s="38"/>
-      <x:c r="C19" s="38"/>
+      <x:c r="C19" s="38" t="str"/>
       <x:c r="D19" s="38"/>
       <x:c r="E19" s="38"/>
       <x:c r="F19" s="38"/>
@@ -1132,11 +1155,12 @@
       <x:c r="P19" s="45"/>
       <x:c r="Q19" s="45"/>
       <x:c r="R19" s="46"/>
+      <x:c r="S19"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="37"/>
       <x:c r="B20" s="38"/>
-      <x:c r="C20" s="38"/>
+      <x:c r="C20" s="38" t="str"/>
       <x:c r="D20" s="38"/>
       <x:c r="E20" s="38"/>
       <x:c r="F20" s="38"/>
@@ -1152,11 +1176,12 @@
       <x:c r="P20" s="45"/>
       <x:c r="Q20" s="45"/>
       <x:c r="R20" s="46"/>
+      <x:c r="S20"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="37"/>
       <x:c r="B21" s="38"/>
-      <x:c r="C21" s="38"/>
+      <x:c r="C21" s="38" t="str"/>
       <x:c r="D21" s="38"/>
       <x:c r="E21" s="38"/>
       <x:c r="F21" s="38"/>
@@ -1172,11 +1197,12 @@
       <x:c r="P21" s="45"/>
       <x:c r="Q21" s="45"/>
       <x:c r="R21" s="46"/>
+      <x:c r="S21"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="37"/>
       <x:c r="B22" s="38"/>
-      <x:c r="C22" s="38"/>
+      <x:c r="C22" s="38" t="str"/>
       <x:c r="D22" s="38"/>
       <x:c r="E22" s="38"/>
       <x:c r="F22" s="38"/>
@@ -1192,11 +1218,12 @@
       <x:c r="P22" s="45"/>
       <x:c r="Q22" s="45"/>
       <x:c r="R22" s="46"/>
+      <x:c r="S22"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="37"/>
       <x:c r="B23" s="38"/>
-      <x:c r="C23" s="38"/>
+      <x:c r="C23" s="38" t="str"/>
       <x:c r="D23" s="38"/>
       <x:c r="E23" s="38"/>
       <x:c r="F23" s="38"/>
@@ -1212,11 +1239,12 @@
       <x:c r="P23" s="45"/>
       <x:c r="Q23" s="45"/>
       <x:c r="R23" s="46"/>
+      <x:c r="S23"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="37"/>
       <x:c r="B24" s="38"/>
-      <x:c r="C24" s="38"/>
+      <x:c r="C24" s="38" t="str"/>
       <x:c r="D24" s="38"/>
       <x:c r="E24" s="38"/>
       <x:c r="F24" s="38"/>
@@ -1232,11 +1260,12 @@
       <x:c r="P24" s="45"/>
       <x:c r="Q24" s="45"/>
       <x:c r="R24" s="46"/>
+      <x:c r="S24"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="37"/>
       <x:c r="B25" s="38"/>
-      <x:c r="C25" s="38"/>
+      <x:c r="C25" s="38" t="str"/>
       <x:c r="D25" s="38"/>
       <x:c r="E25" s="38"/>
       <x:c r="F25" s="38"/>
@@ -1252,11 +1281,12 @@
       <x:c r="P25" s="45"/>
       <x:c r="Q25" s="45"/>
       <x:c r="R25" s="46"/>
+      <x:c r="S25"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="37"/>
       <x:c r="B26" s="38"/>
-      <x:c r="C26" s="38"/>
+      <x:c r="C26" s="38" t="str"/>
       <x:c r="D26" s="38"/>
       <x:c r="E26" s="38"/>
       <x:c r="F26" s="38"/>
@@ -1272,11 +1302,12 @@
       <x:c r="P26" s="45"/>
       <x:c r="Q26" s="45"/>
       <x:c r="R26" s="46"/>
+      <x:c r="S26"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="37"/>
       <x:c r="B27" s="38"/>
-      <x:c r="C27" s="38"/>
+      <x:c r="C27" s="38" t="str"/>
       <x:c r="D27" s="38"/>
       <x:c r="E27" s="38"/>
       <x:c r="F27" s="38"/>
@@ -1292,11 +1323,12 @@
       <x:c r="P27" s="45"/>
       <x:c r="Q27" s="45"/>
       <x:c r="R27" s="46"/>
+      <x:c r="S27"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="37"/>
       <x:c r="B28" s="38"/>
-      <x:c r="C28" s="38"/>
+      <x:c r="C28" s="38" t="str"/>
       <x:c r="D28" s="38"/>
       <x:c r="E28" s="38"/>
       <x:c r="F28" s="38"/>
@@ -1312,11 +1344,12 @@
       <x:c r="P28" s="45"/>
       <x:c r="Q28" s="45"/>
       <x:c r="R28" s="46"/>
+      <x:c r="S28"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="37"/>
       <x:c r="B29" s="38"/>
-      <x:c r="C29" s="38"/>
+      <x:c r="C29" s="38" t="str"/>
       <x:c r="D29" s="38"/>
       <x:c r="E29" s="38"/>
       <x:c r="F29" s="38"/>
@@ -1332,11 +1365,12 @@
       <x:c r="P29" s="45"/>
       <x:c r="Q29" s="45"/>
       <x:c r="R29" s="46"/>
+      <x:c r="S29"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="37"/>
       <x:c r="B30" s="38"/>
-      <x:c r="C30" s="38"/>
+      <x:c r="C30" s="38" t="str"/>
       <x:c r="D30" s="38"/>
       <x:c r="E30" s="38"/>
       <x:c r="F30" s="38"/>
@@ -1352,11 +1386,12 @@
       <x:c r="P30" s="45"/>
       <x:c r="Q30" s="45"/>
       <x:c r="R30" s="46"/>
+      <x:c r="S30"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="37"/>
       <x:c r="B31" s="38"/>
-      <x:c r="C31" s="38"/>
+      <x:c r="C31" s="38" t="str"/>
       <x:c r="D31" s="38"/>
       <x:c r="E31" s="38"/>
       <x:c r="F31" s="38"/>
@@ -1372,11 +1407,12 @@
       <x:c r="P31" s="45"/>
       <x:c r="Q31" s="45"/>
       <x:c r="R31" s="46"/>
+      <x:c r="S31"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="37"/>
       <x:c r="B32" s="38"/>
-      <x:c r="C32" s="38"/>
+      <x:c r="C32" s="38" t="str"/>
       <x:c r="D32" s="38"/>
       <x:c r="E32" s="38"/>
       <x:c r="F32" s="38"/>
@@ -1392,11 +1428,12 @@
       <x:c r="P32" s="45"/>
       <x:c r="Q32" s="45"/>
       <x:c r="R32" s="46"/>
+      <x:c r="S32"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="37"/>
       <x:c r="B33" s="38"/>
-      <x:c r="C33" s="38"/>
+      <x:c r="C33" s="38" t="str"/>
       <x:c r="D33" s="38"/>
       <x:c r="E33" s="38"/>
       <x:c r="F33" s="38"/>
@@ -1412,11 +1449,12 @@
       <x:c r="P33" s="45"/>
       <x:c r="Q33" s="45"/>
       <x:c r="R33" s="46"/>
+      <x:c r="S33"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="37"/>
       <x:c r="B34" s="38"/>
-      <x:c r="C34" s="38"/>
+      <x:c r="C34" s="38" t="str"/>
       <x:c r="D34" s="38"/>
       <x:c r="E34" s="38"/>
       <x:c r="F34" s="38"/>
@@ -1432,11 +1470,12 @@
       <x:c r="P34" s="45"/>
       <x:c r="Q34" s="45"/>
       <x:c r="R34" s="46"/>
+      <x:c r="S34"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="37"/>
       <x:c r="B35" s="38"/>
-      <x:c r="C35" s="38"/>
+      <x:c r="C35" s="38" t="str"/>
       <x:c r="D35" s="38"/>
       <x:c r="E35" s="38"/>
       <x:c r="F35" s="38"/>
@@ -1452,11 +1491,12 @@
       <x:c r="P35" s="45"/>
       <x:c r="Q35" s="45"/>
       <x:c r="R35" s="46"/>
+      <x:c r="S35"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="37"/>
       <x:c r="B36" s="38"/>
-      <x:c r="C36" s="38"/>
+      <x:c r="C36" s="38" t="str"/>
       <x:c r="D36" s="38"/>
       <x:c r="E36" s="38"/>
       <x:c r="F36" s="38"/>
@@ -1472,11 +1512,12 @@
       <x:c r="P36" s="45"/>
       <x:c r="Q36" s="45"/>
       <x:c r="R36" s="46"/>
+      <x:c r="S36"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="37"/>
       <x:c r="B37" s="38"/>
-      <x:c r="C37" s="38"/>
+      <x:c r="C37" s="38" t="str"/>
       <x:c r="D37" s="38"/>
       <x:c r="E37" s="38"/>
       <x:c r="F37" s="38"/>
@@ -1492,11 +1533,12 @@
       <x:c r="P37" s="45"/>
       <x:c r="Q37" s="45"/>
       <x:c r="R37" s="46"/>
+      <x:c r="S37"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="37"/>
       <x:c r="B38" s="38"/>
-      <x:c r="C38" s="38"/>
+      <x:c r="C38" s="38" t="str"/>
       <x:c r="D38" s="38"/>
       <x:c r="E38" s="38"/>
       <x:c r="F38" s="38"/>
@@ -1512,11 +1554,12 @@
       <x:c r="P38" s="45"/>
       <x:c r="Q38" s="45"/>
       <x:c r="R38" s="46"/>
+      <x:c r="S38"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="37"/>
       <x:c r="B39" s="38"/>
-      <x:c r="C39" s="38"/>
+      <x:c r="C39" s="38" t="str"/>
       <x:c r="D39" s="38"/>
       <x:c r="E39" s="38"/>
       <x:c r="F39" s="38"/>
@@ -1532,11 +1575,12 @@
       <x:c r="P39" s="45"/>
       <x:c r="Q39" s="45"/>
       <x:c r="R39" s="46"/>
+      <x:c r="S39"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="37"/>
       <x:c r="B40" s="38"/>
-      <x:c r="C40" s="38"/>
+      <x:c r="C40" s="38" t="str"/>
       <x:c r="D40" s="38"/>
       <x:c r="E40" s="38"/>
       <x:c r="F40" s="38"/>
@@ -1552,11 +1596,12 @@
       <x:c r="P40" s="45"/>
       <x:c r="Q40" s="45"/>
       <x:c r="R40" s="46"/>
+      <x:c r="S40"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="37"/>
       <x:c r="B41" s="38"/>
-      <x:c r="C41" s="38"/>
+      <x:c r="C41" s="38" t="str"/>
       <x:c r="D41" s="38"/>
       <x:c r="E41" s="38"/>
       <x:c r="F41" s="38"/>
@@ -1572,11 +1617,12 @@
       <x:c r="P41" s="45"/>
       <x:c r="Q41" s="45"/>
       <x:c r="R41" s="46"/>
+      <x:c r="S41"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="37"/>
       <x:c r="B42" s="38"/>
-      <x:c r="C42" s="38"/>
+      <x:c r="C42" s="38" t="str"/>
       <x:c r="D42" s="38"/>
       <x:c r="E42" s="38"/>
       <x:c r="F42" s="38"/>
@@ -1592,11 +1638,12 @@
       <x:c r="P42" s="45"/>
       <x:c r="Q42" s="45"/>
       <x:c r="R42" s="46"/>
+      <x:c r="S42"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="37"/>
       <x:c r="B43" s="38"/>
-      <x:c r="C43" s="38"/>
+      <x:c r="C43" s="38" t="str"/>
       <x:c r="D43" s="38"/>
       <x:c r="E43" s="38"/>
       <x:c r="F43" s="38"/>
@@ -1612,11 +1659,12 @@
       <x:c r="P43" s="45"/>
       <x:c r="Q43" s="45"/>
       <x:c r="R43" s="46"/>
+      <x:c r="S43"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="37"/>
       <x:c r="B44" s="38"/>
-      <x:c r="C44" s="38"/>
+      <x:c r="C44" s="38" t="str"/>
       <x:c r="D44" s="38"/>
       <x:c r="E44" s="38"/>
       <x:c r="F44" s="38"/>
@@ -1632,11 +1680,12 @@
       <x:c r="P44" s="45"/>
       <x:c r="Q44" s="45"/>
       <x:c r="R44" s="46"/>
+      <x:c r="S44"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="37"/>
       <x:c r="B45" s="38"/>
-      <x:c r="C45" s="38"/>
+      <x:c r="C45" s="38" t="str"/>
       <x:c r="D45" s="38"/>
       <x:c r="E45" s="38"/>
       <x:c r="F45" s="38"/>
@@ -1652,11 +1701,12 @@
       <x:c r="P45" s="45"/>
       <x:c r="Q45" s="45"/>
       <x:c r="R45" s="46"/>
+      <x:c r="S45"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="37"/>
       <x:c r="B46" s="38"/>
-      <x:c r="C46" s="38"/>
+      <x:c r="C46" s="38" t="str"/>
       <x:c r="D46" s="38"/>
       <x:c r="E46" s="38"/>
       <x:c r="F46" s="38"/>
@@ -1672,11 +1722,12 @@
       <x:c r="P46" s="45"/>
       <x:c r="Q46" s="45"/>
       <x:c r="R46" s="46"/>
+      <x:c r="S46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="37"/>
       <x:c r="B47" s="38"/>
-      <x:c r="C47" s="38"/>
+      <x:c r="C47" s="38" t="str"/>
       <x:c r="D47" s="38"/>
       <x:c r="E47" s="38"/>
       <x:c r="F47" s="38"/>
@@ -1692,11 +1743,12 @@
       <x:c r="P47" s="45"/>
       <x:c r="Q47" s="45"/>
       <x:c r="R47" s="46"/>
+      <x:c r="S47"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="37"/>
       <x:c r="B48" s="38"/>
-      <x:c r="C48" s="38"/>
+      <x:c r="C48" s="38" t="str"/>
       <x:c r="D48" s="38"/>
       <x:c r="E48" s="38"/>
       <x:c r="F48" s="38"/>
@@ -1712,11 +1764,12 @@
       <x:c r="P48" s="45"/>
       <x:c r="Q48" s="45"/>
       <x:c r="R48" s="46"/>
+      <x:c r="S48"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="37"/>
       <x:c r="B49" s="38"/>
-      <x:c r="C49" s="38"/>
+      <x:c r="C49" s="38" t="str"/>
       <x:c r="D49" s="38"/>
       <x:c r="E49" s="38"/>
       <x:c r="F49" s="38"/>
@@ -1732,11 +1785,12 @@
       <x:c r="P49" s="45"/>
       <x:c r="Q49" s="45"/>
       <x:c r="R49" s="46"/>
+      <x:c r="S49"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="37"/>
       <x:c r="B50" s="38"/>
-      <x:c r="C50" s="38"/>
+      <x:c r="C50" s="38" t="str"/>
       <x:c r="D50" s="38"/>
       <x:c r="E50" s="38"/>
       <x:c r="F50" s="38"/>
@@ -1752,11 +1806,12 @@
       <x:c r="P50" s="45"/>
       <x:c r="Q50" s="45"/>
       <x:c r="R50" s="46"/>
+      <x:c r="S50"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="37"/>
       <x:c r="B51" s="38"/>
-      <x:c r="C51" s="38"/>
+      <x:c r="C51" s="38" t="str"/>
       <x:c r="D51" s="38"/>
       <x:c r="E51" s="38"/>
       <x:c r="F51" s="38"/>
@@ -1772,11 +1827,12 @@
       <x:c r="P51" s="45"/>
       <x:c r="Q51" s="45"/>
       <x:c r="R51" s="46"/>
+      <x:c r="S51"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="39"/>
       <x:c r="B52" s="40"/>
-      <x:c r="C52" s="40"/>
+      <x:c r="C52" s="40" t="str"/>
       <x:c r="D52" s="40"/>
       <x:c r="E52" s="40"/>
       <x:c r="F52" s="40"/>
@@ -1792,11 +1848,12 @@
       <x:c r="P52" s="47"/>
       <x:c r="Q52" s="47"/>
       <x:c r="R52" s="48"/>
+      <x:c r="S52"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="41"/>
       <x:c r="B53" s="41"/>
-      <x:c r="C53" s="41"/>
+      <x:c r="C53" s="41" t="str"/>
       <x:c r="D53" s="41"/>
       <x:c r="E53" s="41"/>
       <x:c r="F53" s="41"/>
@@ -1812,11 +1869,12 @@
       <x:c r="P53" s="49"/>
       <x:c r="Q53" s="49"/>
       <x:c r="R53" s="49"/>
+      <x:c r="S53"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="41"/>
       <x:c r="B54" s="41"/>
-      <x:c r="C54" s="41"/>
+      <x:c r="C54" s="41" t="str"/>
       <x:c r="D54" s="41"/>
       <x:c r="E54" s="41"/>
       <x:c r="F54" s="41"/>
@@ -1832,11 +1890,12 @@
       <x:c r="P54" s="49"/>
       <x:c r="Q54" s="49"/>
       <x:c r="R54" s="49"/>
+      <x:c r="S54"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="41"/>
       <x:c r="B55" s="41"/>
-      <x:c r="C55" s="41"/>
+      <x:c r="C55" s="41" t="str"/>
       <x:c r="D55" s="41"/>
       <x:c r="E55" s="41"/>
       <x:c r="F55" s="41"/>
@@ -1852,11 +1911,12 @@
       <x:c r="P55" s="49"/>
       <x:c r="Q55" s="49"/>
       <x:c r="R55" s="49"/>
+      <x:c r="S55"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="41"/>
       <x:c r="B56" s="41"/>
-      <x:c r="C56" s="41"/>
+      <x:c r="C56" s="41" t="str"/>
       <x:c r="D56" s="41"/>
       <x:c r="E56" s="41"/>
       <x:c r="F56" s="41"/>
@@ -1872,11 +1932,12 @@
       <x:c r="P56" s="49"/>
       <x:c r="Q56" s="49"/>
       <x:c r="R56" s="49"/>
+      <x:c r="S56"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="41"/>
       <x:c r="B57" s="41"/>
-      <x:c r="C57" s="41"/>
+      <x:c r="C57" s="41" t="str"/>
       <x:c r="D57" s="41"/>
       <x:c r="E57" s="41"/>
       <x:c r="F57" s="41"/>
@@ -1892,11 +1953,12 @@
       <x:c r="P57" s="49"/>
       <x:c r="Q57" s="49"/>
       <x:c r="R57" s="49"/>
+      <x:c r="S57"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="41"/>
       <x:c r="B58" s="41"/>
-      <x:c r="C58" s="41"/>
+      <x:c r="C58" s="41" t="str"/>
       <x:c r="D58" s="41"/>
       <x:c r="E58" s="41"/>
       <x:c r="F58" s="41"/>
@@ -1912,11 +1974,12 @@
       <x:c r="P58" s="49"/>
       <x:c r="Q58" s="49"/>
       <x:c r="R58" s="49"/>
+      <x:c r="S58"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="41"/>
       <x:c r="B59" s="41"/>
-      <x:c r="C59" s="41"/>
+      <x:c r="C59" s="41" t="str"/>
       <x:c r="D59" s="41"/>
       <x:c r="E59" s="41"/>
       <x:c r="F59" s="41"/>
@@ -1932,11 +1995,12 @@
       <x:c r="P59" s="49"/>
       <x:c r="Q59" s="49"/>
       <x:c r="R59" s="49"/>
+      <x:c r="S59"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="41"/>
       <x:c r="B60" s="41"/>
-      <x:c r="C60" s="41"/>
+      <x:c r="C60" s="41" t="str"/>
       <x:c r="D60" s="41"/>
       <x:c r="E60" s="41"/>
       <x:c r="F60" s="41"/>
@@ -1952,11 +2016,12 @@
       <x:c r="P60" s="49"/>
       <x:c r="Q60" s="49"/>
       <x:c r="R60" s="49"/>
+      <x:c r="S60"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="41"/>
       <x:c r="B61" s="41"/>
-      <x:c r="C61" s="41"/>
+      <x:c r="C61" s="41" t="str"/>
       <x:c r="D61" s="41"/>
       <x:c r="E61" s="41"/>
       <x:c r="F61" s="41"/>
@@ -1972,11 +2037,12 @@
       <x:c r="P61" s="49"/>
       <x:c r="Q61" s="49"/>
       <x:c r="R61" s="49"/>
+      <x:c r="S61"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="41"/>
       <x:c r="B62" s="41"/>
-      <x:c r="C62" s="41"/>
+      <x:c r="C62" s="41" t="str"/>
       <x:c r="D62" s="41"/>
       <x:c r="E62" s="41"/>
       <x:c r="F62" s="41"/>
@@ -1992,11 +2058,12 @@
       <x:c r="P62" s="49"/>
       <x:c r="Q62" s="49"/>
       <x:c r="R62" s="49"/>
+      <x:c r="S62"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="41"/>
       <x:c r="B63" s="41"/>
-      <x:c r="C63" s="41"/>
+      <x:c r="C63" s="41" t="str"/>
       <x:c r="D63" s="41"/>
       <x:c r="E63" s="41"/>
       <x:c r="F63" s="41"/>
@@ -2012,11 +2079,12 @@
       <x:c r="P63" s="49"/>
       <x:c r="Q63" s="49"/>
       <x:c r="R63" s="49"/>
+      <x:c r="S63"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="41"/>
       <x:c r="B64" s="41"/>
-      <x:c r="C64" s="41"/>
+      <x:c r="C64" s="41" t="str"/>
       <x:c r="D64" s="41"/>
       <x:c r="E64" s="41"/>
       <x:c r="F64" s="41"/>
@@ -2032,11 +2100,12 @@
       <x:c r="P64" s="49"/>
       <x:c r="Q64" s="49"/>
       <x:c r="R64" s="49"/>
+      <x:c r="S64"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="41"/>
       <x:c r="B65" s="41"/>
-      <x:c r="C65" s="41"/>
+      <x:c r="C65" s="41" t="str"/>
       <x:c r="D65" s="41"/>
       <x:c r="E65" s="41"/>
       <x:c r="F65" s="41"/>
@@ -2052,11 +2121,12 @@
       <x:c r="P65" s="49"/>
       <x:c r="Q65" s="49"/>
       <x:c r="R65" s="49"/>
+      <x:c r="S65"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="41"/>
       <x:c r="B66" s="41"/>
-      <x:c r="C66" s="41"/>
+      <x:c r="C66" s="41" t="str"/>
       <x:c r="D66" s="41"/>
       <x:c r="E66" s="41"/>
       <x:c r="F66" s="41"/>
@@ -2072,11 +2142,12 @@
       <x:c r="P66" s="49"/>
       <x:c r="Q66" s="49"/>
       <x:c r="R66" s="49"/>
+      <x:c r="S66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="41"/>
       <x:c r="B67" s="41"/>
-      <x:c r="C67" s="41"/>
+      <x:c r="C67" s="41" t="str"/>
       <x:c r="D67" s="41"/>
       <x:c r="E67" s="41"/>
       <x:c r="F67" s="41"/>
@@ -2092,11 +2163,12 @@
       <x:c r="P67" s="49"/>
       <x:c r="Q67" s="49"/>
       <x:c r="R67" s="49"/>
+      <x:c r="S67"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="41"/>
       <x:c r="B68" s="41"/>
-      <x:c r="C68" s="41"/>
+      <x:c r="C68" s="41" t="str"/>
       <x:c r="D68" s="41"/>
       <x:c r="E68" s="41"/>
       <x:c r="F68" s="41"/>
@@ -2112,11 +2184,12 @@
       <x:c r="P68" s="49"/>
       <x:c r="Q68" s="49"/>
       <x:c r="R68" s="49"/>
+      <x:c r="S68"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="41"/>
       <x:c r="B69" s="41"/>
-      <x:c r="C69" s="41"/>
+      <x:c r="C69" s="41" t="str"/>
       <x:c r="D69" s="41"/>
       <x:c r="E69" s="41"/>
       <x:c r="F69" s="41"/>
@@ -2132,11 +2205,12 @@
       <x:c r="P69" s="49"/>
       <x:c r="Q69" s="49"/>
       <x:c r="R69" s="49"/>
+      <x:c r="S69"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="41"/>
       <x:c r="B70" s="41"/>
-      <x:c r="C70" s="41"/>
+      <x:c r="C70" s="41" t="str"/>
       <x:c r="D70" s="41"/>
       <x:c r="E70" s="41"/>
       <x:c r="F70" s="41"/>
@@ -2152,11 +2226,12 @@
       <x:c r="P70" s="49"/>
       <x:c r="Q70" s="49"/>
       <x:c r="R70" s="49"/>
+      <x:c r="S70"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="41"/>
       <x:c r="B71" s="41"/>
-      <x:c r="C71" s="41"/>
+      <x:c r="C71" s="41" t="str"/>
       <x:c r="D71" s="41"/>
       <x:c r="E71" s="41"/>
       <x:c r="F71" s="41"/>
@@ -2172,11 +2247,12 @@
       <x:c r="P71" s="49"/>
       <x:c r="Q71" s="49"/>
       <x:c r="R71" s="49"/>
+      <x:c r="S71"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="41"/>
       <x:c r="B72" s="41"/>
-      <x:c r="C72" s="41"/>
+      <x:c r="C72" s="41" t="str"/>
       <x:c r="D72" s="41"/>
       <x:c r="E72" s="41"/>
       <x:c r="F72" s="41"/>
@@ -2192,11 +2268,12 @@
       <x:c r="P72" s="49"/>
       <x:c r="Q72" s="49"/>
       <x:c r="R72" s="49"/>
+      <x:c r="S72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="41"/>
       <x:c r="B73" s="41"/>
-      <x:c r="C73" s="41"/>
+      <x:c r="C73" s="41" t="str"/>
       <x:c r="D73" s="41"/>
       <x:c r="E73" s="41"/>
       <x:c r="F73" s="41"/>
@@ -2212,11 +2289,12 @@
       <x:c r="P73" s="49"/>
       <x:c r="Q73" s="49"/>
       <x:c r="R73" s="49"/>
+      <x:c r="S73"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="41"/>
       <x:c r="B74" s="41"/>
-      <x:c r="C74" s="41"/>
+      <x:c r="C74" s="41" t="str"/>
       <x:c r="D74" s="41"/>
       <x:c r="E74" s="41"/>
       <x:c r="F74" s="41"/>
@@ -2232,11 +2310,12 @@
       <x:c r="P74" s="49"/>
       <x:c r="Q74" s="49"/>
       <x:c r="R74" s="49"/>
+      <x:c r="S74"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="41"/>
       <x:c r="B75" s="41"/>
-      <x:c r="C75" s="41"/>
+      <x:c r="C75" s="41" t="str"/>
       <x:c r="D75" s="41"/>
       <x:c r="E75" s="41"/>
       <x:c r="F75" s="41"/>
@@ -2252,11 +2331,12 @@
       <x:c r="P75" s="49"/>
       <x:c r="Q75" s="49"/>
       <x:c r="R75" s="49"/>
+      <x:c r="S75"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="41"/>
       <x:c r="B76" s="41"/>
-      <x:c r="C76" s="41"/>
+      <x:c r="C76" s="41" t="str"/>
       <x:c r="D76" s="41"/>
       <x:c r="E76" s="41"/>
       <x:c r="F76" s="41"/>
@@ -2272,11 +2352,12 @@
       <x:c r="P76" s="49"/>
       <x:c r="Q76" s="49"/>
       <x:c r="R76" s="49"/>
+      <x:c r="S76"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="41"/>
       <x:c r="B77" s="41"/>
-      <x:c r="C77" s="41"/>
+      <x:c r="C77" s="41" t="str"/>
       <x:c r="D77" s="41"/>
       <x:c r="E77" s="41"/>
       <x:c r="F77" s="41"/>
@@ -2292,11 +2373,12 @@
       <x:c r="P77" s="49"/>
       <x:c r="Q77" s="49"/>
       <x:c r="R77" s="49"/>
+      <x:c r="S77"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="41"/>
       <x:c r="B78" s="41"/>
-      <x:c r="C78" s="41"/>
+      <x:c r="C78" s="41" t="str"/>
       <x:c r="D78" s="41"/>
       <x:c r="E78" s="41"/>
       <x:c r="F78" s="41"/>
@@ -2312,11 +2394,12 @@
       <x:c r="P78" s="49"/>
       <x:c r="Q78" s="49"/>
       <x:c r="R78" s="49"/>
+      <x:c r="S78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="41"/>
       <x:c r="B79" s="41"/>
-      <x:c r="C79" s="41"/>
+      <x:c r="C79" s="41" t="str"/>
       <x:c r="D79" s="41"/>
       <x:c r="E79" s="41"/>
       <x:c r="F79" s="41"/>
@@ -2332,11 +2415,12 @@
       <x:c r="P79" s="49"/>
       <x:c r="Q79" s="49"/>
       <x:c r="R79" s="49"/>
+      <x:c r="S79"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="41"/>
       <x:c r="B80" s="41"/>
-      <x:c r="C80" s="41"/>
+      <x:c r="C80" s="41" t="str"/>
       <x:c r="D80" s="41"/>
       <x:c r="E80" s="41"/>
       <x:c r="F80" s="41"/>
@@ -2352,11 +2436,12 @@
       <x:c r="P80" s="49"/>
       <x:c r="Q80" s="49"/>
       <x:c r="R80" s="49"/>
+      <x:c r="S80"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="41"/>
       <x:c r="B81" s="41"/>
-      <x:c r="C81" s="41"/>
+      <x:c r="C81" s="41" t="str"/>
       <x:c r="D81" s="41"/>
       <x:c r="E81" s="41"/>
       <x:c r="F81" s="41"/>
@@ -2372,11 +2457,12 @@
       <x:c r="P81" s="49"/>
       <x:c r="Q81" s="49"/>
       <x:c r="R81" s="49"/>
+      <x:c r="S81"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="41"/>
       <x:c r="B82" s="41"/>
-      <x:c r="C82" s="41"/>
+      <x:c r="C82" s="41" t="str"/>
       <x:c r="D82" s="41"/>
       <x:c r="E82" s="41"/>
       <x:c r="F82" s="41"/>
@@ -2392,11 +2478,12 @@
       <x:c r="P82" s="49"/>
       <x:c r="Q82" s="49"/>
       <x:c r="R82" s="49"/>
+      <x:c r="S82"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="41"/>
       <x:c r="B83" s="41"/>
-      <x:c r="C83" s="41"/>
+      <x:c r="C83" s="41" t="str"/>
       <x:c r="D83" s="41"/>
       <x:c r="E83" s="41"/>
       <x:c r="F83" s="41"/>
@@ -2412,11 +2499,12 @@
       <x:c r="P83" s="49"/>
       <x:c r="Q83" s="49"/>
       <x:c r="R83" s="49"/>
+      <x:c r="S83"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="41"/>
       <x:c r="B84" s="41"/>
-      <x:c r="C84" s="41"/>
+      <x:c r="C84" s="41" t="str"/>
       <x:c r="D84" s="41"/>
       <x:c r="E84" s="41"/>
       <x:c r="F84" s="41"/>
@@ -2432,11 +2520,12 @@
       <x:c r="P84" s="49"/>
       <x:c r="Q84" s="49"/>
       <x:c r="R84" s="49"/>
+      <x:c r="S84"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="41"/>
       <x:c r="B85" s="41"/>
-      <x:c r="C85" s="41"/>
+      <x:c r="C85" s="41" t="str"/>
       <x:c r="D85" s="41"/>
       <x:c r="E85" s="41"/>
       <x:c r="F85" s="41"/>
@@ -2452,11 +2541,12 @@
       <x:c r="P85" s="49"/>
       <x:c r="Q85" s="49"/>
       <x:c r="R85" s="49"/>
+      <x:c r="S85"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="41"/>
       <x:c r="B86" s="41"/>
-      <x:c r="C86" s="41"/>
+      <x:c r="C86" s="41" t="str"/>
       <x:c r="D86" s="41"/>
       <x:c r="E86" s="41"/>
       <x:c r="F86" s="41"/>
@@ -2472,11 +2562,12 @@
       <x:c r="P86" s="49"/>
       <x:c r="Q86" s="49"/>
       <x:c r="R86" s="49"/>
+      <x:c r="S86"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="41"/>
       <x:c r="B87" s="41"/>
-      <x:c r="C87" s="41"/>
+      <x:c r="C87" s="41" t="str"/>
       <x:c r="D87" s="41"/>
       <x:c r="E87" s="41"/>
       <x:c r="F87" s="41"/>
@@ -2492,11 +2583,12 @@
       <x:c r="P87" s="49"/>
       <x:c r="Q87" s="49"/>
       <x:c r="R87" s="49"/>
+      <x:c r="S87"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="41"/>
       <x:c r="B88" s="41"/>
-      <x:c r="C88" s="41"/>
+      <x:c r="C88" s="41" t="str"/>
       <x:c r="D88" s="41"/>
       <x:c r="E88" s="41"/>
       <x:c r="F88" s="41"/>
@@ -2512,11 +2604,12 @@
       <x:c r="P88" s="49"/>
       <x:c r="Q88" s="49"/>
       <x:c r="R88" s="49"/>
+      <x:c r="S88"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="41"/>
       <x:c r="B89" s="41"/>
-      <x:c r="C89" s="41"/>
+      <x:c r="C89" s="41" t="str"/>
       <x:c r="D89" s="41"/>
       <x:c r="E89" s="41"/>
       <x:c r="F89" s="41"/>
@@ -2532,11 +2625,12 @@
       <x:c r="P89" s="49"/>
       <x:c r="Q89" s="49"/>
       <x:c r="R89" s="49"/>
+      <x:c r="S89"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="41"/>
       <x:c r="B90" s="41"/>
-      <x:c r="C90" s="41"/>
+      <x:c r="C90" s="41" t="str"/>
       <x:c r="D90" s="41"/>
       <x:c r="E90" s="41"/>
       <x:c r="F90" s="41"/>
@@ -2552,11 +2646,12 @@
       <x:c r="P90" s="49"/>
       <x:c r="Q90" s="49"/>
       <x:c r="R90" s="49"/>
+      <x:c r="S90"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="41"/>
       <x:c r="B91" s="41"/>
-      <x:c r="C91" s="41"/>
+      <x:c r="C91" s="41" t="str"/>
       <x:c r="D91" s="41"/>
       <x:c r="E91" s="41"/>
       <x:c r="F91" s="41"/>
@@ -2572,11 +2667,12 @@
       <x:c r="P91" s="49"/>
       <x:c r="Q91" s="49"/>
       <x:c r="R91" s="49"/>
+      <x:c r="S91"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="41"/>
       <x:c r="B92" s="41"/>
-      <x:c r="C92" s="41"/>
+      <x:c r="C92" s="41" t="str"/>
       <x:c r="D92" s="41"/>
       <x:c r="E92" s="41"/>
       <x:c r="F92" s="41"/>
@@ -2592,11 +2688,12 @@
       <x:c r="P92" s="49"/>
       <x:c r="Q92" s="49"/>
       <x:c r="R92" s="49"/>
+      <x:c r="S92"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="41"/>
       <x:c r="B93" s="41"/>
-      <x:c r="C93" s="41"/>
+      <x:c r="C93" s="41" t="str"/>
       <x:c r="D93" s="41"/>
       <x:c r="E93" s="41"/>
       <x:c r="F93" s="41"/>
@@ -2612,11 +2709,12 @@
       <x:c r="P93" s="49"/>
       <x:c r="Q93" s="49"/>
       <x:c r="R93" s="49"/>
+      <x:c r="S93"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="41"/>
       <x:c r="B94" s="41"/>
-      <x:c r="C94" s="41"/>
+      <x:c r="C94" s="41" t="str"/>
       <x:c r="D94" s="41"/>
       <x:c r="E94" s="41"/>
       <x:c r="F94" s="41"/>
@@ -2632,11 +2730,12 @@
       <x:c r="P94" s="49"/>
       <x:c r="Q94" s="49"/>
       <x:c r="R94" s="49"/>
+      <x:c r="S94"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="41"/>
       <x:c r="B95" s="41"/>
-      <x:c r="C95" s="41"/>
+      <x:c r="C95" s="41" t="str"/>
       <x:c r="D95" s="41"/>
       <x:c r="E95" s="41"/>
       <x:c r="F95" s="41"/>
@@ -2652,11 +2751,12 @@
       <x:c r="P95" s="49"/>
       <x:c r="Q95" s="49"/>
       <x:c r="R95" s="49"/>
+      <x:c r="S95"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="41"/>
       <x:c r="B96" s="41"/>
-      <x:c r="C96" s="41"/>
+      <x:c r="C96" s="41" t="str"/>
       <x:c r="D96" s="41"/>
       <x:c r="E96" s="41"/>
       <x:c r="F96" s="41"/>
@@ -2672,11 +2772,12 @@
       <x:c r="P96" s="49"/>
       <x:c r="Q96" s="49"/>
       <x:c r="R96" s="49"/>
+      <x:c r="S96"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="41"/>
       <x:c r="B97" s="41"/>
-      <x:c r="C97" s="41"/>
+      <x:c r="C97" s="41" t="str"/>
       <x:c r="D97" s="41"/>
       <x:c r="E97" s="41"/>
       <x:c r="F97" s="41"/>
@@ -2692,11 +2793,12 @@
       <x:c r="P97" s="49"/>
       <x:c r="Q97" s="49"/>
       <x:c r="R97" s="49"/>
+      <x:c r="S97"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="41"/>
       <x:c r="B98" s="41"/>
-      <x:c r="C98" s="41"/>
+      <x:c r="C98" s="41" t="str"/>
       <x:c r="D98" s="41"/>
       <x:c r="E98" s="41"/>
       <x:c r="F98" s="41"/>
@@ -2712,11 +2814,12 @@
       <x:c r="P98" s="49"/>
       <x:c r="Q98" s="49"/>
       <x:c r="R98" s="49"/>
+      <x:c r="S98"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="41"/>
       <x:c r="B99" s="41"/>
-      <x:c r="C99" s="41"/>
+      <x:c r="C99" s="41" t="str"/>
       <x:c r="D99" s="41"/>
       <x:c r="E99" s="41"/>
       <x:c r="F99" s="41"/>
@@ -2732,11 +2835,12 @@
       <x:c r="P99" s="49"/>
       <x:c r="Q99" s="49"/>
       <x:c r="R99" s="49"/>
+      <x:c r="S99"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="41"/>
       <x:c r="B100" s="41"/>
-      <x:c r="C100" s="41"/>
+      <x:c r="C100" s="41" t="str"/>
       <x:c r="D100" s="41"/>
       <x:c r="E100" s="41"/>
       <x:c r="F100" s="41"/>
@@ -2752,11 +2856,12 @@
       <x:c r="P100" s="49"/>
       <x:c r="Q100" s="49"/>
       <x:c r="R100" s="49"/>
+      <x:c r="S100"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="41"/>
       <x:c r="B101" s="41"/>
-      <x:c r="C101" s="41"/>
+      <x:c r="C101" s="41" t="str"/>
       <x:c r="D101" s="41"/>
       <x:c r="E101" s="41"/>
       <x:c r="F101" s="41"/>
@@ -2772,11 +2877,12 @@
       <x:c r="P101" s="49"/>
       <x:c r="Q101" s="49"/>
       <x:c r="R101" s="49"/>
+      <x:c r="S101"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="41"/>
       <x:c r="B102" s="41"/>
-      <x:c r="C102" s="41"/>
+      <x:c r="C102" s="41" t="str"/>
       <x:c r="D102" s="41"/>
       <x:c r="E102" s="41"/>
       <x:c r="F102" s="41"/>
@@ -2792,11 +2898,12 @@
       <x:c r="P102" s="49"/>
       <x:c r="Q102" s="49"/>
       <x:c r="R102" s="49"/>
+      <x:c r="S102"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="41"/>
       <x:c r="B103" s="41"/>
-      <x:c r="C103" s="41"/>
+      <x:c r="C103" s="41" t="str"/>
       <x:c r="D103" s="41"/>
       <x:c r="E103" s="41"/>
       <x:c r="F103" s="41"/>
@@ -2812,11 +2919,12 @@
       <x:c r="P103" s="49"/>
       <x:c r="Q103" s="49"/>
       <x:c r="R103" s="49"/>
+      <x:c r="S103"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="41"/>
       <x:c r="B104" s="41"/>
-      <x:c r="C104" s="41"/>
+      <x:c r="C104" s="41" t="str"/>
       <x:c r="D104" s="41"/>
       <x:c r="E104" s="41"/>
       <x:c r="F104" s="41"/>
@@ -2832,11 +2940,12 @@
       <x:c r="P104" s="49"/>
       <x:c r="Q104" s="49"/>
       <x:c r="R104" s="49"/>
+      <x:c r="S104"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="41"/>
       <x:c r="B105" s="41"/>
-      <x:c r="C105" s="41"/>
+      <x:c r="C105" s="41" t="str"/>
       <x:c r="D105" s="41"/>
       <x:c r="E105" s="41"/>
       <x:c r="F105" s="41"/>
@@ -2852,11 +2961,12 @@
       <x:c r="P105" s="49"/>
       <x:c r="Q105" s="49"/>
       <x:c r="R105" s="49"/>
+      <x:c r="S105"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="41"/>
       <x:c r="B106" s="41"/>
-      <x:c r="C106" s="41"/>
+      <x:c r="C106" s="41" t="str"/>
       <x:c r="D106" s="41"/>
       <x:c r="E106" s="41"/>
       <x:c r="F106" s="41"/>
@@ -2872,11 +2982,12 @@
       <x:c r="P106" s="49"/>
       <x:c r="Q106" s="49"/>
       <x:c r="R106" s="49"/>
+      <x:c r="S106"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="41"/>
       <x:c r="B107" s="41"/>
-      <x:c r="C107" s="41"/>
+      <x:c r="C107" s="41" t="str"/>
       <x:c r="D107" s="41"/>
       <x:c r="E107" s="41"/>
       <x:c r="F107" s="41"/>
@@ -2892,11 +3003,12 @@
       <x:c r="P107" s="49"/>
       <x:c r="Q107" s="49"/>
       <x:c r="R107" s="49"/>
+      <x:c r="S107"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="41"/>
       <x:c r="B108" s="41"/>
-      <x:c r="C108" s="41"/>
+      <x:c r="C108" s="41" t="str"/>
       <x:c r="D108" s="41"/>
       <x:c r="E108" s="41"/>
       <x:c r="F108" s="41"/>
@@ -2912,11 +3024,12 @@
       <x:c r="P108" s="49"/>
       <x:c r="Q108" s="49"/>
       <x:c r="R108" s="49"/>
+      <x:c r="S108"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="41"/>
       <x:c r="B109" s="41"/>
-      <x:c r="C109" s="41"/>
+      <x:c r="C109" s="41" t="str"/>
       <x:c r="D109" s="41"/>
       <x:c r="E109" s="41"/>
       <x:c r="F109" s="41"/>
@@ -2932,11 +3045,12 @@
       <x:c r="P109" s="49"/>
       <x:c r="Q109" s="49"/>
       <x:c r="R109" s="49"/>
+      <x:c r="S109"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="41"/>
       <x:c r="B110" s="41"/>
-      <x:c r="C110" s="41"/>
+      <x:c r="C110" s="41" t="str"/>
       <x:c r="D110" s="41"/>
       <x:c r="E110" s="41"/>
       <x:c r="F110" s="41"/>
@@ -2952,11 +3066,12 @@
       <x:c r="P110" s="49"/>
       <x:c r="Q110" s="49"/>
       <x:c r="R110" s="49"/>
+      <x:c r="S110"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="41"/>
       <x:c r="B111" s="41"/>
-      <x:c r="C111" s="41"/>
+      <x:c r="C111" s="41" t="str"/>
       <x:c r="D111" s="41"/>
       <x:c r="E111" s="41"/>
       <x:c r="F111" s="41"/>
@@ -2972,11 +3087,12 @@
       <x:c r="P111" s="49"/>
       <x:c r="Q111" s="49"/>
       <x:c r="R111" s="49"/>
+      <x:c r="S111"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="41"/>
       <x:c r="B112" s="41"/>
-      <x:c r="C112" s="41"/>
+      <x:c r="C112" s="41" t="str"/>
       <x:c r="D112" s="41"/>
       <x:c r="E112" s="41"/>
       <x:c r="F112" s="41"/>
@@ -2992,11 +3108,12 @@
       <x:c r="P112" s="49"/>
       <x:c r="Q112" s="49"/>
       <x:c r="R112" s="49"/>
+      <x:c r="S112"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="41"/>
       <x:c r="B113" s="41"/>
-      <x:c r="C113" s="41"/>
+      <x:c r="C113" s="41" t="str"/>
       <x:c r="D113" s="41"/>
       <x:c r="E113" s="41"/>
       <x:c r="F113" s="41"/>
@@ -3012,11 +3129,12 @@
       <x:c r="P113" s="49"/>
       <x:c r="Q113" s="49"/>
       <x:c r="R113" s="49"/>
+      <x:c r="S113"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="41"/>
       <x:c r="B114" s="41"/>
-      <x:c r="C114" s="41"/>
+      <x:c r="C114" s="41" t="str"/>
       <x:c r="D114" s="41"/>
       <x:c r="E114" s="41"/>
       <x:c r="F114" s="41"/>
@@ -3032,11 +3150,12 @@
       <x:c r="P114" s="49"/>
       <x:c r="Q114" s="49"/>
       <x:c r="R114" s="49"/>
+      <x:c r="S114"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="41"/>
       <x:c r="B115" s="41"/>
-      <x:c r="C115" s="41"/>
+      <x:c r="C115" s="41" t="str"/>
       <x:c r="D115" s="41"/>
       <x:c r="E115" s="41"/>
       <x:c r="F115" s="41"/>
@@ -3052,11 +3171,12 @@
       <x:c r="P115" s="49"/>
       <x:c r="Q115" s="49"/>
       <x:c r="R115" s="49"/>
+      <x:c r="S115"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="41"/>
       <x:c r="B116" s="41"/>
-      <x:c r="C116" s="41"/>
+      <x:c r="C116" s="41" t="str"/>
       <x:c r="D116" s="41"/>
       <x:c r="E116" s="41"/>
       <x:c r="F116" s="41"/>
@@ -3072,11 +3192,12 @@
       <x:c r="P116" s="49"/>
       <x:c r="Q116" s="49"/>
       <x:c r="R116" s="49"/>
+      <x:c r="S116"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="41"/>
       <x:c r="B117" s="41"/>
-      <x:c r="C117" s="41"/>
+      <x:c r="C117" s="41" t="str"/>
       <x:c r="D117" s="41"/>
       <x:c r="E117" s="41"/>
       <x:c r="F117" s="41"/>
@@ -3092,11 +3213,12 @@
       <x:c r="P117" s="49"/>
       <x:c r="Q117" s="49"/>
       <x:c r="R117" s="49"/>
+      <x:c r="S117"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="41"/>
       <x:c r="B118" s="41"/>
-      <x:c r="C118" s="41"/>
+      <x:c r="C118" s="41" t="str"/>
       <x:c r="D118" s="41"/>
       <x:c r="E118" s="41"/>
       <x:c r="F118" s="41"/>
@@ -3112,11 +3234,12 @@
       <x:c r="P118" s="49"/>
       <x:c r="Q118" s="49"/>
       <x:c r="R118" s="49"/>
+      <x:c r="S118"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="41"/>
       <x:c r="B119" s="41"/>
-      <x:c r="C119" s="41"/>
+      <x:c r="C119" s="41" t="str"/>
       <x:c r="D119" s="41"/>
       <x:c r="E119" s="41"/>
       <x:c r="F119" s="41"/>
@@ -3132,11 +3255,12 @@
       <x:c r="P119" s="49"/>
       <x:c r="Q119" s="49"/>
       <x:c r="R119" s="49"/>
+      <x:c r="S119"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="41"/>
       <x:c r="B120" s="41"/>
-      <x:c r="C120" s="41"/>
+      <x:c r="C120" s="41" t="str"/>
       <x:c r="D120" s="41"/>
       <x:c r="E120" s="41"/>
       <x:c r="F120" s="41"/>
@@ -3152,11 +3276,12 @@
       <x:c r="P120" s="49"/>
       <x:c r="Q120" s="49"/>
       <x:c r="R120" s="49"/>
+      <x:c r="S120"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="41"/>
       <x:c r="B121" s="41"/>
-      <x:c r="C121" s="41"/>
+      <x:c r="C121" s="41" t="str"/>
       <x:c r="D121" s="41"/>
       <x:c r="E121" s="41"/>
       <x:c r="F121" s="41"/>
@@ -3172,11 +3297,12 @@
       <x:c r="P121" s="49"/>
       <x:c r="Q121" s="49"/>
       <x:c r="R121" s="49"/>
+      <x:c r="S121"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="41"/>
       <x:c r="B122" s="41"/>
-      <x:c r="C122" s="41"/>
+      <x:c r="C122" s="41" t="str"/>
       <x:c r="D122" s="41"/>
       <x:c r="E122" s="41"/>
       <x:c r="F122" s="41"/>
@@ -3192,11 +3318,12 @@
       <x:c r="P122" s="49"/>
       <x:c r="Q122" s="49"/>
       <x:c r="R122" s="49"/>
+      <x:c r="S122"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="41"/>
       <x:c r="B123" s="41"/>
-      <x:c r="C123" s="41"/>
+      <x:c r="C123" s="41" t="str"/>
       <x:c r="D123" s="41"/>
       <x:c r="E123" s="41"/>
       <x:c r="F123" s="41"/>
@@ -3212,11 +3339,12 @@
       <x:c r="P123" s="49"/>
       <x:c r="Q123" s="49"/>
       <x:c r="R123" s="49"/>
+      <x:c r="S123"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="41"/>
       <x:c r="B124" s="41"/>
-      <x:c r="C124" s="41"/>
+      <x:c r="C124" s="41" t="str"/>
       <x:c r="D124" s="41"/>
       <x:c r="E124" s="41"/>
       <x:c r="F124" s="41"/>
@@ -3232,11 +3360,12 @@
       <x:c r="P124" s="49"/>
       <x:c r="Q124" s="49"/>
       <x:c r="R124" s="49"/>
+      <x:c r="S124"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="41"/>
       <x:c r="B125" s="41"/>
-      <x:c r="C125" s="41"/>
+      <x:c r="C125" s="41" t="str"/>
       <x:c r="D125" s="41"/>
       <x:c r="E125" s="41"/>
       <x:c r="F125" s="41"/>
@@ -3252,11 +3381,12 @@
       <x:c r="P125" s="49"/>
       <x:c r="Q125" s="49"/>
       <x:c r="R125" s="49"/>
+      <x:c r="S125"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="41"/>
       <x:c r="B126" s="41"/>
-      <x:c r="C126" s="41"/>
+      <x:c r="C126" s="41" t="str"/>
       <x:c r="D126" s="41"/>
       <x:c r="E126" s="41"/>
       <x:c r="F126" s="41"/>
@@ -3272,11 +3402,12 @@
       <x:c r="P126" s="49"/>
       <x:c r="Q126" s="49"/>
       <x:c r="R126" s="49"/>
+      <x:c r="S126"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="41"/>
       <x:c r="B127" s="41"/>
-      <x:c r="C127" s="41"/>
+      <x:c r="C127" s="41" t="str"/>
       <x:c r="D127" s="41"/>
       <x:c r="E127" s="41"/>
       <x:c r="F127" s="41"/>
@@ -3292,11 +3423,12 @@
       <x:c r="P127" s="49"/>
       <x:c r="Q127" s="49"/>
       <x:c r="R127" s="49"/>
+      <x:c r="S127"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="41"/>
       <x:c r="B128" s="41"/>
-      <x:c r="C128" s="41"/>
+      <x:c r="C128" s="41" t="str"/>
       <x:c r="D128" s="41"/>
       <x:c r="E128" s="41"/>
       <x:c r="F128" s="41"/>
@@ -3312,11 +3444,12 @@
       <x:c r="P128" s="49"/>
       <x:c r="Q128" s="49"/>
       <x:c r="R128" s="49"/>
+      <x:c r="S128"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="41"/>
       <x:c r="B129" s="41"/>
-      <x:c r="C129" s="41"/>
+      <x:c r="C129" s="41" t="str"/>
       <x:c r="D129" s="41"/>
       <x:c r="E129" s="41"/>
       <x:c r="F129" s="41"/>
@@ -3332,11 +3465,12 @@
       <x:c r="P129" s="49"/>
       <x:c r="Q129" s="49"/>
       <x:c r="R129" s="49"/>
+      <x:c r="S129"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="41"/>
       <x:c r="B130" s="41"/>
-      <x:c r="C130" s="41"/>
+      <x:c r="C130" s="41" t="str"/>
       <x:c r="D130" s="41"/>
       <x:c r="E130" s="41"/>
       <x:c r="F130" s="41"/>
@@ -3352,11 +3486,12 @@
       <x:c r="P130" s="49"/>
       <x:c r="Q130" s="49"/>
       <x:c r="R130" s="49"/>
+      <x:c r="S130"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="41"/>
       <x:c r="B131" s="41"/>
-      <x:c r="C131" s="41"/>
+      <x:c r="C131" s="41" t="str"/>
       <x:c r="D131" s="41"/>
       <x:c r="E131" s="41"/>
       <x:c r="F131" s="41"/>
@@ -3372,11 +3507,12 @@
       <x:c r="P131" s="49"/>
       <x:c r="Q131" s="49"/>
       <x:c r="R131" s="49"/>
+      <x:c r="S131"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="41"/>
       <x:c r="B132" s="41"/>
-      <x:c r="C132" s="41"/>
+      <x:c r="C132" s="41" t="str"/>
       <x:c r="D132" s="41"/>
       <x:c r="E132" s="41"/>
       <x:c r="F132" s="41"/>
@@ -3392,11 +3528,12 @@
       <x:c r="P132" s="49"/>
       <x:c r="Q132" s="49"/>
       <x:c r="R132" s="49"/>
+      <x:c r="S132"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="41"/>
       <x:c r="B133" s="41"/>
-      <x:c r="C133" s="41"/>
+      <x:c r="C133" s="41" t="str"/>
       <x:c r="D133" s="41"/>
       <x:c r="E133" s="41"/>
       <x:c r="F133" s="41"/>
@@ -3412,11 +3549,12 @@
       <x:c r="P133" s="49"/>
       <x:c r="Q133" s="49"/>
       <x:c r="R133" s="49"/>
+      <x:c r="S133"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="41"/>
       <x:c r="B134" s="41"/>
-      <x:c r="C134" s="41"/>
+      <x:c r="C134" s="41" t="str"/>
       <x:c r="D134" s="41"/>
       <x:c r="E134" s="41"/>
       <x:c r="F134" s="41"/>
@@ -3432,11 +3570,12 @@
       <x:c r="P134" s="49"/>
       <x:c r="Q134" s="49"/>
       <x:c r="R134" s="49"/>
+      <x:c r="S134"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="41"/>
       <x:c r="B135" s="41"/>
-      <x:c r="C135" s="41"/>
+      <x:c r="C135" s="41" t="str"/>
       <x:c r="D135" s="41"/>
       <x:c r="E135" s="41"/>
       <x:c r="F135" s="41"/>
@@ -3452,11 +3591,12 @@
       <x:c r="P135" s="49"/>
       <x:c r="Q135" s="49"/>
       <x:c r="R135" s="49"/>
+      <x:c r="S135"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="41"/>
       <x:c r="B136" s="41"/>
-      <x:c r="C136" s="41"/>
+      <x:c r="C136" s="41" t="str"/>
       <x:c r="D136" s="41"/>
       <x:c r="E136" s="41"/>
       <x:c r="F136" s="41"/>
@@ -3472,11 +3612,12 @@
       <x:c r="P136" s="49"/>
       <x:c r="Q136" s="49"/>
       <x:c r="R136" s="49"/>
+      <x:c r="S136"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="41"/>
       <x:c r="B137" s="41"/>
-      <x:c r="C137" s="41"/>
+      <x:c r="C137" s="41" t="str"/>
       <x:c r="D137" s="41"/>
       <x:c r="E137" s="41"/>
       <x:c r="F137" s="41"/>
@@ -3492,11 +3633,12 @@
       <x:c r="P137" s="49"/>
       <x:c r="Q137" s="49"/>
       <x:c r="R137" s="49"/>
+      <x:c r="S137"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="41"/>
       <x:c r="B138" s="41"/>
-      <x:c r="C138" s="41"/>
+      <x:c r="C138" s="41" t="str"/>
       <x:c r="D138" s="41"/>
       <x:c r="E138" s="41"/>
       <x:c r="F138" s="41"/>
@@ -3512,11 +3654,12 @@
       <x:c r="P138" s="49"/>
       <x:c r="Q138" s="49"/>
       <x:c r="R138" s="49"/>
+      <x:c r="S138"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="41"/>
       <x:c r="B139" s="41"/>
-      <x:c r="C139" s="41"/>
+      <x:c r="C139" s="41" t="str"/>
       <x:c r="D139" s="41"/>
       <x:c r="E139" s="41"/>
       <x:c r="F139" s="41"/>
@@ -3532,11 +3675,12 @@
       <x:c r="P139" s="49"/>
       <x:c r="Q139" s="49"/>
       <x:c r="R139" s="49"/>
+      <x:c r="S139"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="41"/>
       <x:c r="B140" s="41"/>
-      <x:c r="C140" s="41"/>
+      <x:c r="C140" s="41" t="str"/>
       <x:c r="D140" s="41"/>
       <x:c r="E140" s="41"/>
       <x:c r="F140" s="41"/>
@@ -3552,11 +3696,12 @@
       <x:c r="P140" s="49"/>
       <x:c r="Q140" s="49"/>
       <x:c r="R140" s="49"/>
+      <x:c r="S140"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="41"/>
       <x:c r="B141" s="41"/>
-      <x:c r="C141" s="41"/>
+      <x:c r="C141" s="41" t="str"/>
       <x:c r="D141" s="41"/>
       <x:c r="E141" s="41"/>
       <x:c r="F141" s="41"/>
@@ -3572,11 +3717,12 @@
       <x:c r="P141" s="49"/>
       <x:c r="Q141" s="49"/>
       <x:c r="R141" s="49"/>
+      <x:c r="S141"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="41"/>
       <x:c r="B142" s="41"/>
-      <x:c r="C142" s="41"/>
+      <x:c r="C142" s="41" t="str"/>
       <x:c r="D142" s="41"/>
       <x:c r="E142" s="41"/>
       <x:c r="F142" s="41"/>
@@ -3592,11 +3738,12 @@
       <x:c r="P142" s="49"/>
       <x:c r="Q142" s="49"/>
       <x:c r="R142" s="49"/>
+      <x:c r="S142"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="41"/>
       <x:c r="B143" s="41"/>
-      <x:c r="C143" s="41"/>
+      <x:c r="C143" s="41" t="str"/>
       <x:c r="D143" s="41"/>
       <x:c r="E143" s="41"/>
       <x:c r="F143" s="41"/>
@@ -3612,11 +3759,12 @@
       <x:c r="P143" s="49"/>
       <x:c r="Q143" s="49"/>
       <x:c r="R143" s="49"/>
+      <x:c r="S143"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="41"/>
       <x:c r="B144" s="41"/>
-      <x:c r="C144" s="41"/>
+      <x:c r="C144" s="41" t="str"/>
       <x:c r="D144" s="41"/>
       <x:c r="E144" s="41"/>
       <x:c r="F144" s="41"/>
@@ -3632,11 +3780,12 @@
       <x:c r="P144" s="49"/>
       <x:c r="Q144" s="49"/>
       <x:c r="R144" s="49"/>
+      <x:c r="S144"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="41"/>
       <x:c r="B145" s="41"/>
-      <x:c r="C145" s="41"/>
+      <x:c r="C145" s="41" t="str"/>
       <x:c r="D145" s="41"/>
       <x:c r="E145" s="41"/>
       <x:c r="F145" s="41"/>
@@ -3652,11 +3801,12 @@
       <x:c r="P145" s="49"/>
       <x:c r="Q145" s="49"/>
       <x:c r="R145" s="49"/>
+      <x:c r="S145"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="41"/>
       <x:c r="B146" s="41"/>
-      <x:c r="C146" s="41"/>
+      <x:c r="C146" s="41" t="str"/>
       <x:c r="D146" s="41"/>
       <x:c r="E146" s="41"/>
       <x:c r="F146" s="41"/>
@@ -3672,11 +3822,12 @@
       <x:c r="P146" s="49"/>
       <x:c r="Q146" s="49"/>
       <x:c r="R146" s="49"/>
+      <x:c r="S146"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="41"/>
       <x:c r="B147" s="41"/>
-      <x:c r="C147" s="41"/>
+      <x:c r="C147" s="41" t="str"/>
       <x:c r="D147" s="41"/>
       <x:c r="E147" s="41"/>
       <x:c r="F147" s="41"/>
@@ -3692,11 +3843,12 @@
       <x:c r="P147" s="49"/>
       <x:c r="Q147" s="49"/>
       <x:c r="R147" s="49"/>
+      <x:c r="S147"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="41"/>
       <x:c r="B148" s="41"/>
-      <x:c r="C148" s="41"/>
+      <x:c r="C148" s="41" t="str"/>
       <x:c r="D148" s="41"/>
       <x:c r="E148" s="41"/>
       <x:c r="F148" s="41"/>
@@ -3712,11 +3864,12 @@
       <x:c r="P148" s="49"/>
       <x:c r="Q148" s="49"/>
       <x:c r="R148" s="49"/>
+      <x:c r="S148"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="41"/>
       <x:c r="B149" s="41"/>
-      <x:c r="C149" s="41"/>
+      <x:c r="C149" s="41" t="str"/>
       <x:c r="D149" s="41"/>
       <x:c r="E149" s="41"/>
       <x:c r="F149" s="41"/>
@@ -3732,11 +3885,12 @@
       <x:c r="P149" s="49"/>
       <x:c r="Q149" s="49"/>
       <x:c r="R149" s="49"/>
+      <x:c r="S149"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="41"/>
       <x:c r="B150" s="41"/>
-      <x:c r="C150" s="41"/>
+      <x:c r="C150" s="41" t="str"/>
       <x:c r="D150" s="41"/>
       <x:c r="E150" s="41"/>
       <x:c r="F150" s="41"/>
@@ -3752,11 +3906,12 @@
       <x:c r="P150" s="49"/>
       <x:c r="Q150" s="49"/>
       <x:c r="R150" s="49"/>
+      <x:c r="S150"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="41"/>
       <x:c r="B151" s="41"/>
-      <x:c r="C151" s="41"/>
+      <x:c r="C151" s="41" t="str"/>
       <x:c r="D151" s="41"/>
       <x:c r="E151" s="41"/>
       <x:c r="F151" s="41"/>
@@ -3772,11 +3927,12 @@
       <x:c r="P151" s="49"/>
       <x:c r="Q151" s="49"/>
       <x:c r="R151" s="49"/>
+      <x:c r="S151"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="41"/>
       <x:c r="B152" s="41"/>
-      <x:c r="C152" s="41"/>
+      <x:c r="C152" s="41" t="str"/>
       <x:c r="D152" s="41"/>
       <x:c r="E152" s="41"/>
       <x:c r="F152" s="41"/>
@@ -3792,11 +3948,12 @@
       <x:c r="P152" s="49"/>
       <x:c r="Q152" s="49"/>
       <x:c r="R152" s="49"/>
+      <x:c r="S152"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="41"/>
       <x:c r="B153" s="41"/>
-      <x:c r="C153" s="41"/>
+      <x:c r="C153" s="41" t="str"/>
       <x:c r="D153" s="41"/>
       <x:c r="E153" s="41"/>
       <x:c r="F153" s="41"/>
@@ -3812,11 +3969,12 @@
       <x:c r="P153" s="49"/>
       <x:c r="Q153" s="49"/>
       <x:c r="R153" s="49"/>
+      <x:c r="S153"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="41"/>
       <x:c r="B154" s="41"/>
-      <x:c r="C154" s="41"/>
+      <x:c r="C154" s="41" t="str"/>
       <x:c r="D154" s="41"/>
       <x:c r="E154" s="41"/>
       <x:c r="F154" s="41"/>
@@ -3832,11 +3990,12 @@
       <x:c r="P154" s="49"/>
       <x:c r="Q154" s="49"/>
       <x:c r="R154" s="49"/>
+      <x:c r="S154"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="41"/>
       <x:c r="B155" s="41"/>
-      <x:c r="C155" s="41"/>
+      <x:c r="C155" s="41" t="str"/>
       <x:c r="D155" s="41"/>
       <x:c r="E155" s="41"/>
       <x:c r="F155" s="41"/>
@@ -3852,11 +4011,12 @@
       <x:c r="P155" s="49"/>
       <x:c r="Q155" s="49"/>
       <x:c r="R155" s="49"/>
+      <x:c r="S155"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="41"/>
       <x:c r="B156" s="41"/>
-      <x:c r="C156" s="41"/>
+      <x:c r="C156" s="41" t="str"/>
       <x:c r="D156" s="41"/>
       <x:c r="E156" s="41"/>
       <x:c r="F156" s="41"/>
@@ -3872,11 +4032,12 @@
       <x:c r="P156" s="49"/>
       <x:c r="Q156" s="49"/>
       <x:c r="R156" s="49"/>
+      <x:c r="S156"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="41"/>
       <x:c r="B157" s="41"/>
-      <x:c r="C157" s="41"/>
+      <x:c r="C157" s="41" t="str"/>
       <x:c r="D157" s="41"/>
       <x:c r="E157" s="41"/>
       <x:c r="F157" s="41"/>
@@ -3892,11 +4053,12 @@
       <x:c r="P157" s="49"/>
       <x:c r="Q157" s="49"/>
       <x:c r="R157" s="49"/>
+      <x:c r="S157"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="41"/>
       <x:c r="B158" s="41"/>
-      <x:c r="C158" s="41"/>
+      <x:c r="C158" s="41" t="str"/>
       <x:c r="D158" s="41"/>
       <x:c r="E158" s="41"/>
       <x:c r="F158" s="41"/>
@@ -3912,11 +4074,12 @@
       <x:c r="P158" s="49"/>
       <x:c r="Q158" s="49"/>
       <x:c r="R158" s="49"/>
+      <x:c r="S158"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="41"/>
       <x:c r="B159" s="41"/>
-      <x:c r="C159" s="41"/>
+      <x:c r="C159" s="41" t="str"/>
       <x:c r="D159" s="41"/>
       <x:c r="E159" s="41"/>
       <x:c r="F159" s="41"/>
@@ -3932,11 +4095,12 @@
       <x:c r="P159" s="49"/>
       <x:c r="Q159" s="49"/>
       <x:c r="R159" s="49"/>
+      <x:c r="S159"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="41"/>
       <x:c r="B160" s="41"/>
-      <x:c r="C160" s="41"/>
+      <x:c r="C160" s="41" t="str"/>
       <x:c r="D160" s="41"/>
       <x:c r="E160" s="41"/>
       <x:c r="F160" s="41"/>
@@ -3952,11 +4116,12 @@
       <x:c r="P160" s="49"/>
       <x:c r="Q160" s="49"/>
       <x:c r="R160" s="49"/>
+      <x:c r="S160"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="41"/>
       <x:c r="B161" s="41"/>
-      <x:c r="C161" s="41"/>
+      <x:c r="C161" s="41" t="str"/>
       <x:c r="D161" s="41"/>
       <x:c r="E161" s="41"/>
       <x:c r="F161" s="41"/>
@@ -3972,11 +4137,12 @@
       <x:c r="P161" s="49"/>
       <x:c r="Q161" s="49"/>
       <x:c r="R161" s="49"/>
+      <x:c r="S161"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="41"/>
       <x:c r="B162" s="41"/>
-      <x:c r="C162" s="41"/>
+      <x:c r="C162" s="41" t="str"/>
       <x:c r="D162" s="41"/>
       <x:c r="E162" s="41"/>
       <x:c r="F162" s="41"/>
@@ -3992,11 +4158,12 @@
       <x:c r="P162" s="49"/>
       <x:c r="Q162" s="49"/>
       <x:c r="R162" s="49"/>
+      <x:c r="S162"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="41"/>
       <x:c r="B163" s="41"/>
-      <x:c r="C163" s="41"/>
+      <x:c r="C163" s="41" t="str"/>
       <x:c r="D163" s="41"/>
       <x:c r="E163" s="41"/>
       <x:c r="F163" s="41"/>
@@ -4012,11 +4179,12 @@
       <x:c r="P163" s="49"/>
       <x:c r="Q163" s="49"/>
       <x:c r="R163" s="49"/>
+      <x:c r="S163"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="41"/>
       <x:c r="B164" s="41"/>
-      <x:c r="C164" s="41"/>
+      <x:c r="C164" s="41" t="str"/>
       <x:c r="D164" s="41"/>
       <x:c r="E164" s="41"/>
       <x:c r="F164" s="41"/>
@@ -4032,11 +4200,12 @@
       <x:c r="P164" s="49"/>
       <x:c r="Q164" s="49"/>
       <x:c r="R164" s="49"/>
+      <x:c r="S164"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="41"/>
       <x:c r="B165" s="41"/>
-      <x:c r="C165" s="41"/>
+      <x:c r="C165" s="41" t="str"/>
       <x:c r="D165" s="41"/>
       <x:c r="E165" s="41"/>
       <x:c r="F165" s="41"/>
@@ -4052,11 +4221,12 @@
       <x:c r="P165" s="49"/>
       <x:c r="Q165" s="49"/>
       <x:c r="R165" s="49"/>
+      <x:c r="S165"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="41"/>
       <x:c r="B166" s="41"/>
-      <x:c r="C166" s="41"/>
+      <x:c r="C166" s="41" t="str"/>
       <x:c r="D166" s="41"/>
       <x:c r="E166" s="41"/>
       <x:c r="F166" s="41"/>
@@ -4072,11 +4242,12 @@
       <x:c r="P166" s="49"/>
       <x:c r="Q166" s="49"/>
       <x:c r="R166" s="49"/>
+      <x:c r="S166"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="41"/>
       <x:c r="B167" s="41"/>
-      <x:c r="C167" s="41"/>
+      <x:c r="C167" s="41" t="str"/>
       <x:c r="D167" s="41"/>
       <x:c r="E167" s="41"/>
       <x:c r="F167" s="41"/>
@@ -4092,11 +4263,12 @@
       <x:c r="P167" s="49"/>
       <x:c r="Q167" s="49"/>
       <x:c r="R167" s="49"/>
+      <x:c r="S167"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="41"/>
       <x:c r="B168" s="41"/>
-      <x:c r="C168" s="41"/>
+      <x:c r="C168" s="41" t="str"/>
       <x:c r="D168" s="41"/>
       <x:c r="E168" s="41"/>
       <x:c r="F168" s="41"/>
@@ -4112,11 +4284,12 @@
       <x:c r="P168" s="49"/>
       <x:c r="Q168" s="49"/>
       <x:c r="R168" s="49"/>
+      <x:c r="S168"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="41"/>
       <x:c r="B169" s="41"/>
-      <x:c r="C169" s="41"/>
+      <x:c r="C169" s="41" t="str"/>
       <x:c r="D169" s="41"/>
       <x:c r="E169" s="41"/>
       <x:c r="F169" s="41"/>
@@ -4132,11 +4305,12 @@
       <x:c r="P169" s="49"/>
       <x:c r="Q169" s="49"/>
       <x:c r="R169" s="49"/>
+      <x:c r="S169"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="41"/>
       <x:c r="B170" s="41"/>
-      <x:c r="C170" s="41"/>
+      <x:c r="C170" s="41" t="str"/>
       <x:c r="D170" s="41"/>
       <x:c r="E170" s="41"/>
       <x:c r="F170" s="41"/>
@@ -4152,11 +4326,12 @@
       <x:c r="P170" s="49"/>
       <x:c r="Q170" s="49"/>
       <x:c r="R170" s="49"/>
+      <x:c r="S170"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="41"/>
       <x:c r="B171" s="41"/>
-      <x:c r="C171" s="41"/>
+      <x:c r="C171" s="41" t="str"/>
       <x:c r="D171" s="41"/>
       <x:c r="E171" s="41"/>
       <x:c r="F171" s="41"/>
@@ -4172,11 +4347,12 @@
       <x:c r="P171" s="49"/>
       <x:c r="Q171" s="49"/>
       <x:c r="R171" s="49"/>
+      <x:c r="S171"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="41"/>
       <x:c r="B172" s="41"/>
-      <x:c r="C172" s="41"/>
+      <x:c r="C172" s="41" t="str"/>
       <x:c r="D172" s="41"/>
       <x:c r="E172" s="41"/>
       <x:c r="F172" s="41"/>
@@ -4192,11 +4368,12 @@
       <x:c r="P172" s="49"/>
       <x:c r="Q172" s="49"/>
       <x:c r="R172" s="49"/>
+      <x:c r="S172"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="41"/>
       <x:c r="B173" s="41"/>
-      <x:c r="C173" s="41"/>
+      <x:c r="C173" s="41" t="str"/>
       <x:c r="D173" s="41"/>
       <x:c r="E173" s="41"/>
       <x:c r="F173" s="41"/>
@@ -4212,11 +4389,12 @@
       <x:c r="P173" s="49"/>
       <x:c r="Q173" s="49"/>
       <x:c r="R173" s="49"/>
+      <x:c r="S173"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="41"/>
       <x:c r="B174" s="41"/>
-      <x:c r="C174" s="41"/>
+      <x:c r="C174" s="41" t="str"/>
       <x:c r="D174" s="41"/>
       <x:c r="E174" s="41"/>
       <x:c r="F174" s="41"/>
@@ -4232,11 +4410,12 @@
       <x:c r="P174" s="49"/>
       <x:c r="Q174" s="49"/>
       <x:c r="R174" s="49"/>
+      <x:c r="S174"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="41"/>
       <x:c r="B175" s="41"/>
-      <x:c r="C175" s="41"/>
+      <x:c r="C175" s="41" t="str"/>
       <x:c r="D175" s="41"/>
       <x:c r="E175" s="41"/>
       <x:c r="F175" s="41"/>
@@ -4252,11 +4431,12 @@
       <x:c r="P175" s="49"/>
       <x:c r="Q175" s="49"/>
       <x:c r="R175" s="49"/>
+      <x:c r="S175"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="41"/>
       <x:c r="B176" s="41"/>
-      <x:c r="C176" s="41"/>
+      <x:c r="C176" s="41" t="str"/>
       <x:c r="D176" s="41"/>
       <x:c r="E176" s="41"/>
       <x:c r="F176" s="41"/>
@@ -4272,11 +4452,12 @@
       <x:c r="P176" s="49"/>
       <x:c r="Q176" s="49"/>
       <x:c r="R176" s="49"/>
+      <x:c r="S176"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="41"/>
       <x:c r="B177" s="41"/>
-      <x:c r="C177" s="41"/>
+      <x:c r="C177" s="41" t="str"/>
       <x:c r="D177" s="41"/>
       <x:c r="E177" s="41"/>
       <x:c r="F177" s="41"/>
@@ -4292,11 +4473,12 @@
       <x:c r="P177" s="49"/>
       <x:c r="Q177" s="49"/>
       <x:c r="R177" s="49"/>
+      <x:c r="S177"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="41"/>
       <x:c r="B178" s="41"/>
-      <x:c r="C178" s="41"/>
+      <x:c r="C178" s="41" t="str"/>
       <x:c r="D178" s="41"/>
       <x:c r="E178" s="41"/>
       <x:c r="F178" s="41"/>
@@ -4312,11 +4494,12 @@
       <x:c r="P178" s="49"/>
       <x:c r="Q178" s="49"/>
       <x:c r="R178" s="49"/>
+      <x:c r="S178"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="41"/>
       <x:c r="B179" s="41"/>
-      <x:c r="C179" s="41"/>
+      <x:c r="C179" s="41" t="str"/>
       <x:c r="D179" s="41"/>
       <x:c r="E179" s="41"/>
       <x:c r="F179" s="41"/>
@@ -4332,11 +4515,12 @@
       <x:c r="P179" s="49"/>
       <x:c r="Q179" s="49"/>
       <x:c r="R179" s="49"/>
+      <x:c r="S179"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="41"/>
       <x:c r="B180" s="41"/>
-      <x:c r="C180" s="41"/>
+      <x:c r="C180" s="41" t="str"/>
       <x:c r="D180" s="41"/>
       <x:c r="E180" s="41"/>
       <x:c r="F180" s="41"/>
@@ -4352,11 +4536,12 @@
       <x:c r="P180" s="49"/>
       <x:c r="Q180" s="49"/>
       <x:c r="R180" s="49"/>
+      <x:c r="S180"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="41"/>
       <x:c r="B181" s="41"/>
-      <x:c r="C181" s="41"/>
+      <x:c r="C181" s="41" t="str"/>
       <x:c r="D181" s="41"/>
       <x:c r="E181" s="41"/>
       <x:c r="F181" s="41"/>
@@ -4372,11 +4557,12 @@
       <x:c r="P181" s="49"/>
       <x:c r="Q181" s="49"/>
       <x:c r="R181" s="49"/>
+      <x:c r="S181"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="41"/>
       <x:c r="B182" s="41"/>
-      <x:c r="C182" s="41"/>
+      <x:c r="C182" s="41" t="str"/>
       <x:c r="D182" s="41"/>
       <x:c r="E182" s="41"/>
       <x:c r="F182" s="41"/>
@@ -4392,11 +4578,12 @@
       <x:c r="P182" s="49"/>
       <x:c r="Q182" s="49"/>
       <x:c r="R182" s="49"/>
+      <x:c r="S182"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="41"/>
       <x:c r="B183" s="41"/>
-      <x:c r="C183" s="41"/>
+      <x:c r="C183" s="41" t="str"/>
       <x:c r="D183" s="41"/>
       <x:c r="E183" s="41"/>
       <x:c r="F183" s="41"/>
@@ -4412,11 +4599,12 @@
       <x:c r="P183" s="49"/>
       <x:c r="Q183" s="49"/>
       <x:c r="R183" s="49"/>
+      <x:c r="S183"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="41"/>
       <x:c r="B184" s="41"/>
-      <x:c r="C184" s="41"/>
+      <x:c r="C184" s="41" t="str"/>
       <x:c r="D184" s="41"/>
       <x:c r="E184" s="41"/>
       <x:c r="F184" s="41"/>
@@ -4432,11 +4620,12 @@
       <x:c r="P184" s="49"/>
       <x:c r="Q184" s="49"/>
       <x:c r="R184" s="49"/>
+      <x:c r="S184"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="41"/>
       <x:c r="B185" s="41"/>
-      <x:c r="C185" s="41"/>
+      <x:c r="C185" s="41" t="str"/>
       <x:c r="D185" s="41"/>
       <x:c r="E185" s="41"/>
       <x:c r="F185" s="41"/>
@@ -4452,11 +4641,12 @@
       <x:c r="P185" s="49"/>
       <x:c r="Q185" s="49"/>
       <x:c r="R185" s="49"/>
+      <x:c r="S185"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="41"/>
       <x:c r="B186" s="41"/>
-      <x:c r="C186" s="41"/>
+      <x:c r="C186" s="41" t="str"/>
       <x:c r="D186" s="41"/>
       <x:c r="E186" s="41"/>
       <x:c r="F186" s="41"/>
@@ -4472,11 +4662,12 @@
       <x:c r="P186" s="49"/>
       <x:c r="Q186" s="49"/>
       <x:c r="R186" s="49"/>
+      <x:c r="S186"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="41"/>
       <x:c r="B187" s="41"/>
-      <x:c r="C187" s="41"/>
+      <x:c r="C187" s="41" t="str"/>
       <x:c r="D187" s="41"/>
       <x:c r="E187" s="41"/>
       <x:c r="F187" s="41"/>
@@ -4492,11 +4683,12 @@
       <x:c r="P187" s="49"/>
       <x:c r="Q187" s="49"/>
       <x:c r="R187" s="49"/>
+      <x:c r="S187"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="41"/>
       <x:c r="B188" s="41"/>
-      <x:c r="C188" s="41"/>
+      <x:c r="C188" s="41" t="str"/>
       <x:c r="D188" s="41"/>
       <x:c r="E188" s="41"/>
       <x:c r="F188" s="41"/>
@@ -4512,11 +4704,12 @@
       <x:c r="P188" s="49"/>
       <x:c r="Q188" s="49"/>
       <x:c r="R188" s="49"/>
+      <x:c r="S188"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="41"/>
       <x:c r="B189" s="41"/>
-      <x:c r="C189" s="41"/>
+      <x:c r="C189" s="41" t="str"/>
       <x:c r="D189" s="41"/>
       <x:c r="E189" s="41"/>
       <x:c r="F189" s="41"/>
@@ -4532,11 +4725,12 @@
       <x:c r="P189" s="49"/>
       <x:c r="Q189" s="49"/>
       <x:c r="R189" s="49"/>
+      <x:c r="S189"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="41"/>
       <x:c r="B190" s="41"/>
-      <x:c r="C190" s="41"/>
+      <x:c r="C190" s="41" t="str"/>
       <x:c r="D190" s="41"/>
       <x:c r="E190" s="41"/>
       <x:c r="F190" s="41"/>
@@ -4552,11 +4746,12 @@
       <x:c r="P190" s="49"/>
       <x:c r="Q190" s="49"/>
       <x:c r="R190" s="49"/>
+      <x:c r="S190"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="41"/>
       <x:c r="B191" s="41"/>
-      <x:c r="C191" s="41"/>
+      <x:c r="C191" s="41" t="str"/>
       <x:c r="D191" s="41"/>
       <x:c r="E191" s="41"/>
       <x:c r="F191" s="41"/>
@@ -4572,11 +4767,12 @@
       <x:c r="P191" s="49"/>
       <x:c r="Q191" s="49"/>
       <x:c r="R191" s="49"/>
+      <x:c r="S191"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="41"/>
       <x:c r="B192" s="41"/>
-      <x:c r="C192" s="41"/>
+      <x:c r="C192" s="41" t="str"/>
       <x:c r="D192" s="41"/>
       <x:c r="E192" s="41"/>
       <x:c r="F192" s="41"/>
@@ -4592,11 +4788,12 @@
       <x:c r="P192" s="49"/>
       <x:c r="Q192" s="49"/>
       <x:c r="R192" s="49"/>
+      <x:c r="S192"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="41"/>
       <x:c r="B193" s="41"/>
-      <x:c r="C193" s="41"/>
+      <x:c r="C193" s="41" t="str"/>
       <x:c r="D193" s="41"/>
       <x:c r="E193" s="41"/>
       <x:c r="F193" s="41"/>
@@ -4612,11 +4809,12 @@
       <x:c r="P193" s="49"/>
       <x:c r="Q193" s="49"/>
       <x:c r="R193" s="49"/>
+      <x:c r="S193"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="41"/>
       <x:c r="B194" s="41"/>
-      <x:c r="C194" s="41"/>
+      <x:c r="C194" s="41" t="str"/>
       <x:c r="D194" s="41"/>
       <x:c r="E194" s="41"/>
       <x:c r="F194" s="41"/>
@@ -4632,11 +4830,12 @@
       <x:c r="P194" s="49"/>
       <x:c r="Q194" s="49"/>
       <x:c r="R194" s="49"/>
+      <x:c r="S194"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="41"/>
       <x:c r="B195" s="41"/>
-      <x:c r="C195" s="41"/>
+      <x:c r="C195" s="41" t="str"/>
       <x:c r="D195" s="41"/>
       <x:c r="E195" s="41"/>
       <x:c r="F195" s="41"/>
@@ -4652,11 +4851,12 @@
       <x:c r="P195" s="49"/>
       <x:c r="Q195" s="49"/>
       <x:c r="R195" s="49"/>
+      <x:c r="S195"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="41"/>
       <x:c r="B196" s="41"/>
-      <x:c r="C196" s="41"/>
+      <x:c r="C196" s="41" t="str"/>
       <x:c r="D196" s="41"/>
       <x:c r="E196" s="41"/>
       <x:c r="F196" s="41"/>
@@ -4672,11 +4872,12 @@
       <x:c r="P196" s="49"/>
       <x:c r="Q196" s="49"/>
       <x:c r="R196" s="49"/>
+      <x:c r="S196"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="41"/>
       <x:c r="B197" s="41"/>
-      <x:c r="C197" s="41"/>
+      <x:c r="C197" s="41" t="str"/>
       <x:c r="D197" s="41"/>
       <x:c r="E197" s="41"/>
       <x:c r="F197" s="41"/>
@@ -4692,11 +4893,12 @@
       <x:c r="P197" s="49"/>
       <x:c r="Q197" s="49"/>
       <x:c r="R197" s="49"/>
+      <x:c r="S197"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="41"/>
       <x:c r="B198" s="41"/>
-      <x:c r="C198" s="41"/>
+      <x:c r="C198" s="41" t="str"/>
       <x:c r="D198" s="41"/>
       <x:c r="E198" s="41"/>
       <x:c r="F198" s="41"/>
@@ -4712,11 +4914,12 @@
       <x:c r="P198" s="49"/>
       <x:c r="Q198" s="49"/>
       <x:c r="R198" s="49"/>
+      <x:c r="S198"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="41"/>
       <x:c r="B199" s="41"/>
-      <x:c r="C199" s="41"/>
+      <x:c r="C199" s="41" t="str"/>
       <x:c r="D199" s="41"/>
       <x:c r="E199" s="41"/>
       <x:c r="F199" s="41"/>
@@ -4732,11 +4935,12 @@
       <x:c r="P199" s="49"/>
       <x:c r="Q199" s="49"/>
       <x:c r="R199" s="49"/>
+      <x:c r="S199"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="41"/>
       <x:c r="B200" s="41"/>
-      <x:c r="C200" s="41"/>
+      <x:c r="C200" s="41" t="str"/>
       <x:c r="D200" s="41"/>
       <x:c r="E200" s="41"/>
       <x:c r="F200" s="41"/>
@@ -4752,6 +4956,7 @@
       <x:c r="P200" s="49"/>
       <x:c r="Q200" s="49"/>
       <x:c r="R200" s="49"/>
+      <x:c r="S200"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -4761,7 +4966,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6b46cea049b4f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb786c2e3db1c4a1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>